<commit_message>
fix(autopageMKII): identify SKUs still missing SN via red-alert btn-serial on POS when qty matches but SMCO requests serial
</commit_message>
<xml_diff>
--- a/projects/auto_page/autopageMKII/tables/Accel_mode_uat.xlsx
+++ b/projects/auto_page/autopageMKII/tables/Accel_mode_uat.xlsx
@@ -653,11 +653,7 @@
       <c r="C26" s="7" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="inlineStr">
-        <is>
-          <t>260805HCA5Y6XM</t>
-        </is>
-      </c>
+      <c r="A27" s="7" t="inlineStr"/>
       <c r="B27" s="7" t="inlineStr"/>
       <c r="C27" s="7" t="inlineStr"/>
     </row>
@@ -770,11 +766,7 @@
       <c r="C39" s="7" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="7" t="inlineStr">
-        <is>
-          <t>260805H97WNP8E</t>
-        </is>
-      </c>
+      <c r="A40" s="7" t="inlineStr"/>
       <c r="B40" s="7" t="inlineStr"/>
       <c r="C40" s="7" t="inlineStr"/>
     </row>
@@ -815,11 +807,7 @@
       <c r="C44" s="7" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
-        <is>
-          <t>260805HA9UW4U4</t>
-        </is>
-      </c>
+      <c r="A45" s="7" t="inlineStr"/>
       <c r="B45" s="7" t="inlineStr"/>
       <c r="C45" s="7" t="inlineStr"/>
     </row>
@@ -833,38 +821,22 @@
       <c r="C46" s="7" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="7" t="inlineStr">
-        <is>
-          <t>260805H9EYP2T3</t>
-        </is>
-      </c>
+      <c r="A47" s="7" t="inlineStr"/>
       <c r="B47" s="7" t="inlineStr"/>
       <c r="C47" s="7" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="7" t="inlineStr">
-        <is>
-          <t>260805H9GAN62D</t>
-        </is>
-      </c>
+      <c r="A48" s="7" t="inlineStr"/>
       <c r="B48" s="7" t="inlineStr"/>
       <c r="C48" s="7" t="inlineStr"/>
     </row>
     <row r="49">
-      <c r="A49" s="7" t="inlineStr">
-        <is>
-          <t>260805H7NMUJJU</t>
-        </is>
-      </c>
+      <c r="A49" s="7" t="inlineStr"/>
       <c r="B49" s="7" t="inlineStr"/>
       <c r="C49" s="7" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="7" t="inlineStr">
-        <is>
-          <t>260805H98W4V8D</t>
-        </is>
-      </c>
+      <c r="A50" s="7" t="inlineStr"/>
       <c r="B50" s="7" t="inlineStr"/>
       <c r="C50" s="7" t="inlineStr"/>
     </row>
@@ -887,11 +859,7 @@
       <c r="C52" s="7" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="7" t="inlineStr">
-        <is>
-          <t>260805H6DEAUGS</t>
-        </is>
-      </c>
+      <c r="A53" s="7" t="inlineStr"/>
       <c r="B53" s="7" t="inlineStr"/>
       <c r="C53" s="7" t="inlineStr"/>
     </row>
@@ -6277,7 +6245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C458"/>
+  <dimension ref="A1:C480"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15885,6 +15853,463 @@
         </is>
       </c>
     </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>260805HD001FB8</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not found for SKU: PR5-000658 (วันที่: 2026-08-05 10:01, ราคาที่ต้องออกบิล: 3478.0)
+SHOPEE เวลาสั่งซื้อ 2026-08-05 10:01
+PR5-000658 BROTHER DCP-T230 ปริ้นเตอร์ (PR5-000658)
+ยิงขายขึ้น 4,290.00 บาท
+ลูกค้าซื้อราคา 3,478.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:12:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>260805HCH35X3F</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>ไม่มีสินค้าให้ตรวจสอบและปรับราคา สำหรับ SKU: MNL-002091 (วันที่: 2026-08-05 09:52, ราคาที่ต้องออกบิล: 3137.0) (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:13:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>260805HC3K7A6J</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not found for SKU: SP4-000196 (วันที่: 2026-08-05 09:45, ราคาที่ต้องออกบิล: 315.0)
+SHOPEE เวลาสั่งซื้อ 2026-08-05 09:45
+SP4-000196 Epson EPS RB S015582/S015306 LQ630 หมึกพิมพ์ (SP4-000196)
+ยิงขายขึ้น 320.00 บาท
+ลูกค้าซื้อราคา 315.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:13:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>260805HC9PQH5N</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not found for SKU: SP4-000302 (วันที่: 2026-08-05 09:48, ราคาที่ต้องออกบิล: 143.0)
+SHOPEE เวลาสั่งซื้อ 2026-08-05 09:48
+SP4-000302 Epson RB S015639/LQ-310 (SP4-000302)  ตลับผ้าหมึก
+ยิงขายขึ้น 150.00 บาท
+ลูกค้าซื้อราคา 143.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:14:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>260805HC39KTHC</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not found for SKU: SP2-001703+SP2-001596+SP2-001597+SP2-001598 (วันที่: 2026-08-05 09:45, ราคาที่ต้องออกบิล: 981.0)
+SHOPEE เวลาสั่งซื้อ 2026-08-05 09:45
+SP2-001703+SP2-001596+SP2-001597+SP2-001598 Brother หมึกเติมของแท้รุ่น BT-D60BK,5000C,M,Y และ PACK 4 สี
+ยิงขายขึ้น 1,030.00 บาท
+ลูกค้าซื้อราคา 981.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:14:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>260805HAAKR17H</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not found for SKU: MNL-002514 (วันที่: 2026-08-05 09:13, ราคาที่ต้องออกบิล: 5605.0)
+SHOPEE เวลาสั่งซื้อ 2026-08-05 09:13
+MNL-002514 LENOVO Legion Gaming Monitor 27Q-10 - 27"/2K/IPS/240Hz/0.5ms/NVIDIA G-SYNC Compatible AMD FreeSync Premium/ MNL-002514
+ยิงขายขึ้น 6,591.00 บาท
+ลูกค้าซื้อราคา 5,605.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:15:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>260805HBTN1VNH</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>please input serial.
+⚠️ SKU ทั้งหมดลงบน POS ครบแล้ว แต่ SMCO ยังขอ serial (ตรวจสอบ SN ที่กรอกด้วยมือ) (ด่านที่ติด: กรอก Skus ลง POS)</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:15:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>260805HBND8HM7</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>please input serial.
+⚠️ SKU ทั้งหมดลงบน POS ครบแล้ว แต่ SMCO ยังขอ serial (ตรวจสอบ SN ที่กรอกด้วยมือ) (ด่านที่ติด: กรอก Skus ลง POS)</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:16:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>260805HBE1NGH6</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not found for SKU: PR5-000582 (วันที่: 2026-08-05 09:33, ราคาที่ต้องออกบิล: 2256.0)
+SHOPEE เวลาสั่งซื้อ 2026-08-05 09:33
+PR5-000582 Canon เครื่องพิมพ์อิงค์เจ็ท PIXMA รุ่น E3370 Printer *พร้อมหมึกแท้ในกล่อง 1 ชุด*(PR5-000582)
+ยิงขายขึ้น 3,490.00 บาท
+ลูกค้าซื้อราคา 2,256.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:16:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>260805H8YV5CVH</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not found for SKU: MNL-002409 (วันที่: 2026-08-05 08:49, ราคาที่ต้องออกบิล: 2852.0)
+SHOPEE เวลาสั่งซื้อ 2026-08-05 08:49
+MNL-002409 MSI Monitor PRO MP241W E14V - 23.8"/VA/144Hz/1ms/Adaptive-Sync/3Y*3(White) MNL-002409
+ยิงขายขึ้น 2,923.00 บาท
+ลูกค้าซื้อราคา 2,852.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:17:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>260805HBBGK4WC</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not found for SKU: PR5-000646 (วันที่: 2026-08-05 09:31, ราคาที่ต้องออกบิล: 4647.0)
+SHOPEE เวลาสั่งซื้อ 2026-08-05 09:31
+PR5-000646 Canon เครื่องพิมพ์อิงค์เจ็ท PIXMA รุ่น G3730 (2Y)*พร้อมหมึกแท้ในกล่อง 1 ชุด*
+ยิงขายขึ้น 5,590.00 บาท
+ลูกค้าซื้อราคา 4,647.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:17:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>260805HB8WKTXU</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>please input serial.
+⚠️ SKU ทั้งหมดลงบน POS ครบแล้ว แต่ SMCO ยังขอ serial (ตรวจสอบ SN ที่กรอกด้วยมือ) (ด่านที่ติด: กรอก Skus ลง POS)</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:17:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>260805HB2S6M9U</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not found for SKU: OE3-000289 (วันที่: 2026-08-05 09:27, ราคาที่ต้องออกบิล: 759.0)
+SHOPEE เวลาสั่งซื้อ 2026-08-05 09:27
+OE3-000289 LOGITECH HEADSET H390 USB COMPUTER  (2Y)
+ยิงขายขึ้น 999.00 บาท
+ลูกค้าซื้อราคา 759.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:18:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>260805H9CPA5X4</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not found for SKU: SP2-001792+SP2-001793+SP2-001794+SP2-001795 (วันที่: 2026-08-05 08:56, ราคาที่ต้องออกบิล: 1386.0)
+SHOPEE เวลาสั่งซื้อ 2026-08-05 08:56
+SP2-001792+SP2-001793+SP2-001794+SP2-001795 Canon ตลับหมึกอิงค์เจ็ท รุ่น GI 71 BK / C / M / Y และ PACK 4 สี
+ยิงขายขึ้น 1,600.00 บาท
+ลูกค้าซื้อราคา 1,386.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:18:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>260805HAU517DM</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not found for SKU: MNL-001886 (วันที่: 2026-08-05 09:22, ราคาที่ต้องออกบิล: 5929.0)
+SHOPEE เวลาสั่งซื้อ 2026-08-05 09:22
+MNL-001886 DAHUA Gaming Monitor Curved LM30-E330C - 30"/VA/WFHD/200Hz/1ms/Adaptive Sync/3Y*3 (Black)  MNL-001886
+ยิงขายขึ้น 7,713.00 บาท
+ลูกค้าซื้อราคา 5,929.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:19:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>260805H95FH9WB</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>ราคา/จำนวนไม่ตรงหลังปรับราคา: SKU Price mismatch: SP2-001713+SP2-001714+SP2-001715+SP2-001716 (expected 1213.0, actual 1252.0, diff -39.0) | Total Price mismatch (expected 1213.0, actual 1252.0)
+SHOPEE เวลาสั่งซื้อ 2026-08-05 08:52
+SP2-001713+SP2-001714+SP2-001715+SP2-001716 Epson หมึกแท้รุ่น T00V (003) Ink Bottle BK / C / M / Y และ PACK 4 สี
+ยิงขายขึ้น 1,252.00 บาท
+ลูกค้าซื้อราคา 1,213.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ปรับราคา/ใส่คูปองสำเร็จ (จบ process ปรับราคา))</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:19:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>260805HASCT1PN</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not found for SKU: MNL-002519 (วันที่: 2026-08-05 09:21, ราคาที่ต้องออกบิล: 3436.0)
+SHOPEE เวลาสั่งซื้อ 2026-08-05 09:21
+MNL-002519 ASUS TUF Gaming Monitor VG259QM5A - 24.5"/IPS/240Hz/0.3ms/FreeSync Premium, G-Sync Compatible/3Y*3 MNL-002519
+ยิงขายขึ้น 3,712.00 บาท
+ลูกค้าซื้อราคา 3,436.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:20:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>260805H8TFKXJX</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not found for SKU: SP2-001610+SP2-001611+SP2-001612+SP2-001613 (วันที่: 2026-08-05 08:46, ราคาที่ต้องออกบิล: 1211.0)
+SHOPEE เวลาสั่งซื้อ 2026-08-05 08:46
+SP2-001610+SP2-001611+SP2-001612+SP2-001613 Canon หมึกอิงค์เจ็ท รุ่น GI 790 BK / C / M / Y และ PACK 4 สี
+ยิงขายขึ้น 1,280.00 บาท
+ลูกค้าซื้อราคา 1,211.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:20:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>260805H80F15F4</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not found for SKU: SP4-000302 (วันที่: 2026-08-05 08:32, ราคาที่ต้องออกบิล: 143.0)
+SHOPEE เวลาสั่งซื้อ 2026-08-05 08:32
+SP4-000302 Epson RB S015639/LQ-310 (SP4-000302)  ตลับผ้าหมึก
+ยิงขายขึ้น 150.00 บาท
+ลูกค้าซื้อราคา 143.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:21:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>260805GHMUCBF0</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>ไม่พบออเดอร์ 260805GHMUCBF0 ในระบบ Shopee หรือค้นหาไม่สำเร็จ (ด่านที่ติด: เริ่มรัน)</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:21:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>260805H76N3T6T</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Order skipped, CP/DC not found for SKU: MNL-002519 (วันที่: 2026-08-05 08:17, ราคาที่ต้องออกบิล: 3436.0)
+SHOPEE เวลาสั่งซื้อ 2026-08-05 08:17
+MNL-002519 ASUS TUF Gaming Monitor VG259QM5A - 24.5"/IPS/240Hz/0.3ms/FreeSync Premium, G-Sync Compatible/3Y*3 MNL-002519
+ยิงขายขึ้น 3,712.00 บาท
+ลูกค้าซื้อราคา 3,436.00 บาท
+ขอวิธีปรับราคาครับ (ด่านที่ติด: ตรวจสอบราคาและจำนวนสำเร็จ)</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:22:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>260805H6B5U5FN</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>ไม่พบออเดอร์ 260805H6B5U5FN ในระบบ Shopee หรือค้นหาไม่สำเร็จ (ด่านที่ติด: เริ่มรัน)</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:22:22</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15896,7 +16321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17664,6 +18089,166 @@
       <c r="F87" s="7" t="inlineStr">
         <is>
           <t>2026-08-05 17:11:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="7" t="inlineStr"/>
+      <c r="B88" s="7" t="inlineStr">
+        <is>
+          <t>260805HCA5Y6XM</t>
+        </is>
+      </c>
+      <c r="C88" s="7" t="inlineStr"/>
+      <c r="D88" s="7" t="inlineStr"/>
+      <c r="E88" s="7" t="inlineStr">
+        <is>
+          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
+        </is>
+      </c>
+      <c r="F88" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:13:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="7" t="inlineStr"/>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>260805H97WNP8E</t>
+        </is>
+      </c>
+      <c r="C89" s="7" t="inlineStr"/>
+      <c r="D89" s="7" t="inlineStr"/>
+      <c r="E89" s="7" t="inlineStr">
+        <is>
+          <t>ข้าม (สถานะ: ยกเลิกแล้ว)</t>
+        </is>
+      </c>
+      <c r="F89" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:18:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="7" t="inlineStr"/>
+      <c r="B90" s="7" t="inlineStr">
+        <is>
+          <t>260805HA9UW4U4</t>
+        </is>
+      </c>
+      <c r="C90" s="7" t="inlineStr"/>
+      <c r="D90" s="7" t="inlineStr"/>
+      <c r="E90" s="7" t="inlineStr">
+        <is>
+          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
+        </is>
+      </c>
+      <c r="F90" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:20:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="7" t="inlineStr"/>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>260805H9EYP2T3</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="inlineStr"/>
+      <c r="D91" s="7" t="inlineStr"/>
+      <c r="E91" s="7" t="inlineStr">
+        <is>
+          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
+        </is>
+      </c>
+      <c r="F91" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:21:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="7" t="inlineStr"/>
+      <c r="B92" s="7" t="inlineStr">
+        <is>
+          <t>260805H9GAN62D</t>
+        </is>
+      </c>
+      <c r="C92" s="7" t="inlineStr"/>
+      <c r="D92" s="7" t="inlineStr"/>
+      <c r="E92" s="7" t="inlineStr">
+        <is>
+          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
+        </is>
+      </c>
+      <c r="F92" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:21:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="7" t="inlineStr"/>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>260805H7NMUJJU</t>
+        </is>
+      </c>
+      <c r="C93" s="7" t="inlineStr"/>
+      <c r="D93" s="7" t="inlineStr"/>
+      <c r="E93" s="7" t="inlineStr">
+        <is>
+          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
+        </is>
+      </c>
+      <c r="F93" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:21:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="7" t="inlineStr"/>
+      <c r="B94" s="7" t="inlineStr">
+        <is>
+          <t>260805H98W4V8D</t>
+        </is>
+      </c>
+      <c r="C94" s="7" t="inlineStr"/>
+      <c r="D94" s="7" t="inlineStr"/>
+      <c r="E94" s="7" t="inlineStr">
+        <is>
+          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
+        </is>
+      </c>
+      <c r="F94" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:21:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="7" t="inlineStr"/>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>260805H6DEAUGS</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="inlineStr"/>
+      <c r="D95" s="7" t="inlineStr"/>
+      <c r="E95" s="7" t="inlineStr">
+        <is>
+          <t>ข้าม (สถานะ: ส่งสินค้าแล้ว)</t>
+        </is>
+      </c>
+      <c r="F95" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-05 17:22:17</t>
         </is>
       </c>
     </row>

</xml_diff>